<commit_message>
new changes made in the UI for the pratice section
</commit_message>
<xml_diff>
--- a/public/templates/all_questions_template.xlsx
+++ b/public/templates/all_questions_template.xlsx
@@ -397,19 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="50.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="80.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:P11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,6 +430,24 @@
       <c r="J1" t="str">
         <v>Test Cases JSON</v>
       </c>
+      <c r="K1" t="str">
+        <v>Difficulty</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Concept</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Company Name</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Exam Name</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Exam Year</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Section Name</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -474,6 +480,24 @@
       <c r="J2" t="str">
         <v/>
       </c>
+      <c r="K2" t="str">
+        <v>easy</v>
+      </c>
+      <c r="L2" t="str">
+        <v>programming</v>
+      </c>
+      <c r="M2" t="str">
+        <v>tcs</v>
+      </c>
+      <c r="N2" t="str">
+        <v>nqt</v>
+      </c>
+      <c r="O2" t="str">
+        <v>2025</v>
+      </c>
+      <c r="P2" t="str">
+        <v>coding</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -506,6 +530,24 @@
       <c r="J3" t="str">
         <v/>
       </c>
+      <c r="K3" t="str">
+        <v>medium</v>
+      </c>
+      <c r="L3" t="str">
+        <v>logical</v>
+      </c>
+      <c r="M3" t="str">
+        <v>infosys, wipro</v>
+      </c>
+      <c r="N3" t="str">
+        <v>infytq, wiprotest</v>
+      </c>
+      <c r="O3" t="str">
+        <v>2025, 2026</v>
+      </c>
+      <c r="P3" t="str">
+        <v>coding, technical</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -538,6 +580,24 @@
       <c r="J4" t="str">
         <v/>
       </c>
+      <c r="K4" t="str">
+        <v>hard</v>
+      </c>
+      <c r="L4" t="str">
+        <v>math</v>
+      </c>
+      <c r="M4" t="str">
+        <v>cognizant</v>
+      </c>
+      <c r="N4" t="str">
+        <v>genC</v>
+      </c>
+      <c r="O4" t="str">
+        <v>2026</v>
+      </c>
+      <c r="P4" t="str">
+        <v>logical</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -570,6 +630,24 @@
       <c r="J5" t="str">
         <v/>
       </c>
+      <c r="K5" t="str">
+        <v>medium</v>
+      </c>
+      <c r="L5" t="str">
+        <v>fundamentals</v>
+      </c>
+      <c r="M5" t="str">
+        <v>amazon</v>
+      </c>
+      <c r="N5" t="str">
+        <v>aws-cert</v>
+      </c>
+      <c r="O5" t="str">
+        <v>2024</v>
+      </c>
+      <c r="P5" t="str">
+        <v>verbal</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -602,6 +680,24 @@
       <c r="J6" t="str">
         <v/>
       </c>
+      <c r="K6" t="str">
+        <v>easy</v>
+      </c>
+      <c r="L6" t="str">
+        <v>science</v>
+      </c>
+      <c r="M6" t="str">
+        <v>google, microsoft</v>
+      </c>
+      <c r="N6" t="str">
+        <v>g-kickstart, ms-codility</v>
+      </c>
+      <c r="O6" t="str">
+        <v>2024, 2025</v>
+      </c>
+      <c r="P6" t="str">
+        <v>algorithms, technical</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -634,6 +730,24 @@
       <c r="J7" t="str">
         <v/>
       </c>
+      <c r="K7" t="str">
+        <v>easy</v>
+      </c>
+      <c r="L7" t="str">
+        <v>programming</v>
+      </c>
+      <c r="M7" t="str">
+        <v>tcs</v>
+      </c>
+      <c r="N7" t="str">
+        <v>nqt</v>
+      </c>
+      <c r="O7" t="str">
+        <v>2025</v>
+      </c>
+      <c r="P7" t="str">
+        <v>coding</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -666,6 +780,24 @@
       <c r="J8" t="str">
         <v/>
       </c>
+      <c r="K8" t="str">
+        <v>medium</v>
+      </c>
+      <c r="L8" t="str">
+        <v>logical</v>
+      </c>
+      <c r="M8" t="str">
+        <v>infosys, wipro</v>
+      </c>
+      <c r="N8" t="str">
+        <v>infytq, wiprotest</v>
+      </c>
+      <c r="O8" t="str">
+        <v>2025, 2026</v>
+      </c>
+      <c r="P8" t="str">
+        <v>coding, technical</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -698,6 +830,24 @@
       <c r="J9" t="str">
         <v/>
       </c>
+      <c r="K9" t="str">
+        <v>hard</v>
+      </c>
+      <c r="L9" t="str">
+        <v>math</v>
+      </c>
+      <c r="M9" t="str">
+        <v>cognizant</v>
+      </c>
+      <c r="N9" t="str">
+        <v>genC</v>
+      </c>
+      <c r="O9" t="str">
+        <v>2026</v>
+      </c>
+      <c r="P9" t="str">
+        <v>logical</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -730,6 +880,24 @@
       <c r="J10" t="str">
         <v>[{"input":"2, 3","expectedOutput":"5","explanation":"2 + 3 = 5"},{"input":"10, 20","expectedOutput":"30","explanation":"10 + 20 = 30"}]</v>
       </c>
+      <c r="K10" t="str">
+        <v>medium</v>
+      </c>
+      <c r="L10" t="str">
+        <v>fundamentals</v>
+      </c>
+      <c r="M10" t="str">
+        <v>amazon</v>
+      </c>
+      <c r="N10" t="str">
+        <v>aws-cert</v>
+      </c>
+      <c r="O10" t="str">
+        <v>2024</v>
+      </c>
+      <c r="P10" t="str">
+        <v>verbal</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -762,10 +930,28 @@
       <c r="J11" t="str">
         <v>[{"input":"4","expectedOutput":"true","explanation":"4 is divisible by 2"},{"input":"7","expectedOutput":"false","explanation":"7 is not divisible by 2"}]</v>
       </c>
+      <c r="K11" t="str">
+        <v>easy</v>
+      </c>
+      <c r="L11" t="str">
+        <v>science</v>
+      </c>
+      <c r="M11" t="str">
+        <v>google, microsoft</v>
+      </c>
+      <c r="N11" t="str">
+        <v>g-kickstart, ms-codility</v>
+      </c>
+      <c r="O11" t="str">
+        <v>2024, 2025</v>
+      </c>
+      <c r="P11" t="str">
+        <v>algorithms, technical</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>